<commit_message>
Rebuild 動画配信 templates on 19期 第1回 full body
Replaced the minimal placeholder 動画配信 templates with the full 19期
第1回 mail structure. 第1回 keeps the オリエンテーション block; 第2〜6
open with a shorter greeting. Per-lecture parts (title, video list,
task list including ブログチャレンジ / インスタチャレンジ) are marked
"（ここに追記）" for the user to fill per row. Also swaps the 課題提出先リンク
line for {{課題提出先リンクまとめ}} — a new 基本設定 key so the URL is
shared across all six lectures instead of pasted six times.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019MpwpoXeU7u2s8oySrLx9o
</commit_message>
<xml_diff>
--- a/scratchpad/MailTemplates_20ki_v2.xlsx
+++ b/scratchpad/MailTemplates_20ki_v2.xlsx
@@ -1379,24 +1379,60 @@
           <t>※このメールは、『{{期}}期"Shine A Light"』の皆さまにお送りしております。
 こんにちは
 Shine A Light 運営事務局です。
-本日、第1回目の講義動画を会員サイトにアップいたしました。
+いよいよ本日より第1回目の講義動画配信がスタートいたします。
+3ヶ月、どうぞよろしくお願いいたします！
+【第1回目の動画講義のご案内】
+第1回目の講義動画を会員サイトにアップしました。
+会員サイトよりご視聴ください。
+まずは、オリエンテーションからご確認ください。
+＝＝＝＝＝＝＝＝＝
+オリエンテーション
+"Shine A Light"の進め方説明動画（52分）
+（オリエンテーション動画URLをここに追記）
+＝＝＝＝＝＝＝＝＝
+※講義動画を視聴する前にご視聴ください
+《内容》
+①MVV（ミッション、ヴィジョン、ヴァリュー）
+②会員サイトの使い方
+③事前準備チェックシート
+④自己コーチングシート入力について
+⑤連絡方法メッセンジャーグループの使い方
+⑥講座専用FBグループの使い方
+⑦バディ制度と週報について
+⑧課題の提出方法
+⑨士業相談について
 ＝＝＝＝＝＝＝
+第1回目講義動画「（講義タイトルをここに入れる）」
+＝＝＝＝＝＝＝
+会員サイトよりご視聴ください。
+モジュールの項目で第1回目の講義動画をご視聴可能です。
 {{会員サイト}}
-＝＝＝＝＝＝＝
-第1回目の講義動画をご視聴ください。
-＜第1回目:ブランディング＞
-(動画本数・内容の詳細は、下書きに直接追記してください)
+＜第1回目の内容：（講義タイトル）＞
+（動画本数：X本）
+（動画①のタイトル（分）をここに追記）
+（動画②のタイトル（分））
+（動画③...）
+＜第1回目課題まとめは以下になります＞
+（課題①をここに追記）
+（課題② ※ブログチャレンジ、インスタチャレンジ等もここに）
+（課題③）
+講義動画ご視聴後は、
+{{期}}期のFBグループに第1回目講義のまとめも必ずご覧ください
 ━━━━━━━━━━━━━━━━━━━━━━
-【要挿入:Facebook投稿リンク】
-下記3つのFB投稿リンクを、送信前に貼り付けてください
+【要挿入：Facebook投稿リンク】
+下記2つのFB投稿リンクを、送信前に貼り付けてください
 ▼第1回目講義まとめ
-(URL挿入)
+（URL挿入）
 ▼課題をこなすための動画リンクなど
-(URL挿入)
-▼課題提出先リンクまとめ
-(URL挿入)
+（URL挿入）
 ━━━━━━━━━━━━━━━━━━━━━━
+【課題提出先リンクまとめ】
+{{課題提出先リンクまとめ}}
+※ご自身のお名前のシートをご自由にご活用ください。
 課題提出の期限は次回の講義動画配信日までとなっております。
+【次回の講座のグルコンの予定】
+（次回のグルコン予定をここに追記）
+ぜひご参加ください。
 ご案内は以上です。
 ご不明点のお問い合わせは
 当メールの返信にてご連絡ください。
@@ -1426,24 +1462,42 @@
           <t>※このメールは、『{{期}}期"Shine A Light"』の皆さまにお送りしております。
 こんにちは
 Shine A Light 運営事務局です。
-本日、第2回目の講義動画を会員サイトにアップいたしました。
+本日、第2回目の講義動画をお届けいたします。
+【第2回目の動画講義のご案内】
+第2回目の講義動画を会員サイトにアップしました。
+会員サイトよりご視聴ください。
 ＝＝＝＝＝＝＝
+第2回目講義動画「（講義タイトルをここに入れる）」
+＝＝＝＝＝＝＝
+会員サイトよりご視聴ください。
+モジュールの項目で第2回目の講義動画をご視聴可能です。
 {{会員サイト}}
-＝＝＝＝＝＝＝
-第2回目の講義動画をご視聴ください。
-＜第2回目:商品設計＞
-(動画本数・内容の詳細は、下書きに直接追記してください)
+＜第2回目の内容：（講義タイトル）＞
+（動画本数：X本）
+（動画①のタイトル（分）をここに追記）
+（動画②のタイトル（分））
+（動画③...）
+＜第2回目課題まとめは以下になります＞
+（課題①をここに追記）
+（課題② ※ブログチャレンジ、インスタチャレンジ等もここに）
+（課題③）
+講義動画ご視聴後は、
+{{期}}期のFBグループに第2回目講義のまとめも必ずご覧ください
 ━━━━━━━━━━━━━━━━━━━━━━
-【要挿入:Facebook投稿リンク】
-下記3つのFB投稿リンクを、送信前に貼り付けてください
+【要挿入：Facebook投稿リンク】
+下記2つのFB投稿リンクを、送信前に貼り付けてください
 ▼第2回目講義まとめ
-(URL挿入)
+（URL挿入）
 ▼課題をこなすための動画リンクなど
-(URL挿入)
-▼課題提出先リンクまとめ
-(URL挿入)
+（URL挿入）
 ━━━━━━━━━━━━━━━━━━━━━━
+【課題提出先リンクまとめ】
+{{課題提出先リンクまとめ}}
+※ご自身のお名前のシートをご自由にご活用ください。
 課題提出の期限は次回の講義動画配信日までとなっております。
+【次回の講座のグルコンの予定】
+（次回のグルコン予定をここに追記）
+ぜひご参加ください。
 ご案内は以上です。
 ご不明点のお問い合わせは
 当メールの返信にてご連絡ください。
@@ -1473,24 +1527,42 @@
           <t>※このメールは、『{{期}}期"Shine A Light"』の皆さまにお送りしております。
 こんにちは
 Shine A Light 運営事務局です。
-本日、第3回目の講義動画を会員サイトにアップいたしました。
+本日、第3回目の講義動画をお届けいたします。
+【第3回目の動画講義のご案内】
+第3回目の講義動画を会員サイトにアップしました。
+会員サイトよりご視聴ください。
 ＝＝＝＝＝＝＝
+第3回目講義動画「（講義タイトルをここに入れる）」
+＝＝＝＝＝＝＝
+会員サイトよりご視聴ください。
+モジュールの項目で第3回目の講義動画をご視聴可能です。
 {{会員サイト}}
-＝＝＝＝＝＝＝
-第3回目の講義動画をご視聴ください。
-＜第3回目:集客・SNS＞
-(動画本数・内容の詳細は、下書きに直接追記してください)
+＜第3回目の内容：（講義タイトル）＞
+（動画本数：X本）
+（動画①のタイトル（分）をここに追記）
+（動画②のタイトル（分））
+（動画③...）
+＜第3回目課題まとめは以下になります＞
+（課題①をここに追記）
+（課題② ※ブログチャレンジ、インスタチャレンジ等もここに）
+（課題③）
+講義動画ご視聴後は、
+{{期}}期のFBグループに第3回目講義のまとめも必ずご覧ください
 ━━━━━━━━━━━━━━━━━━━━━━
-【要挿入:Facebook投稿リンク】
-下記3つのFB投稿リンクを、送信前に貼り付けてください
+【要挿入：Facebook投稿リンク】
+下記2つのFB投稿リンクを、送信前に貼り付けてください
 ▼第3回目講義まとめ
-(URL挿入)
+（URL挿入）
 ▼課題をこなすための動画リンクなど
-(URL挿入)
-▼課題提出先リンクまとめ
-(URL挿入)
+（URL挿入）
 ━━━━━━━━━━━━━━━━━━━━━━
+【課題提出先リンクまとめ】
+{{課題提出先リンクまとめ}}
+※ご自身のお名前のシートをご自由にご活用ください。
 課題提出の期限は次回の講義動画配信日までとなっております。
+【次回の講座のグルコンの予定】
+（次回のグルコン予定をここに追記）
+ぜひご参加ください。
 ご案内は以上です。
 ご不明点のお問い合わせは
 当メールの返信にてご連絡ください。
@@ -1520,24 +1592,42 @@
           <t>※このメールは、『{{期}}期"Shine A Light"』の皆さまにお送りしております。
 こんにちは
 Shine A Light 運営事務局です。
-本日、第4回目の講義動画を会員サイトにアップいたしました。
+本日、第4回目の講義動画をお届けいたします。
+【第4回目の動画講義のご案内】
+第4回目の講義動画を会員サイトにアップしました。
+会員サイトよりご視聴ください。
 ＝＝＝＝＝＝＝
+第4回目講義動画「（講義タイトルをここに入れる）」
+＝＝＝＝＝＝＝
+会員サイトよりご視聴ください。
+モジュールの項目で第4回目の講義動画をご視聴可能です。
 {{会員サイト}}
-＝＝＝＝＝＝＝
-第4回目の講義動画をご視聴ください。
-＜第4回目:セールス＞
-(動画本数・内容の詳細は、下書きに直接追記してください)
+＜第4回目の内容：（講義タイトル）＞
+（動画本数：X本）
+（動画①のタイトル（分）をここに追記）
+（動画②のタイトル（分））
+（動画③...）
+＜第4回目課題まとめは以下になります＞
+（課題①をここに追記）
+（課題② ※ブログチャレンジ、インスタチャレンジ等もここに）
+（課題③）
+講義動画ご視聴後は、
+{{期}}期のFBグループに第4回目講義のまとめも必ずご覧ください
 ━━━━━━━━━━━━━━━━━━━━━━
-【要挿入:Facebook投稿リンク】
-下記3つのFB投稿リンクを、送信前に貼り付けてください
+【要挿入：Facebook投稿リンク】
+下記2つのFB投稿リンクを、送信前に貼り付けてください
 ▼第4回目講義まとめ
-(URL挿入)
+（URL挿入）
 ▼課題をこなすための動画リンクなど
-(URL挿入)
-▼課題提出先リンクまとめ
-(URL挿入)
+（URL挿入）
 ━━━━━━━━━━━━━━━━━━━━━━
+【課題提出先リンクまとめ】
+{{課題提出先リンクまとめ}}
+※ご自身のお名前のシートをご自由にご活用ください。
 課題提出の期限は次回の講義動画配信日までとなっております。
+【次回の講座のグルコンの予定】
+（次回のグルコン予定をここに追記）
+ぜひご参加ください。
 ご案内は以上です。
 ご不明点のお問い合わせは
 当メールの返信にてご連絡ください。
@@ -1567,24 +1657,42 @@
           <t>※このメールは、『{{期}}期"Shine A Light"』の皆さまにお送りしております。
 こんにちは
 Shine A Light 運営事務局です。
-本日、第5回目の講義動画を会員サイトにアップいたしました。
+本日、第5回目の講義動画をお届けいたします。
+【第5回目の動画講義のご案内】
+第5回目の講義動画を会員サイトにアップしました。
+会員サイトよりご視聴ください。
 ＝＝＝＝＝＝＝
+第5回目講義動画「（講義タイトルをここに入れる）」
+＝＝＝＝＝＝＝
+会員サイトよりご視聴ください。
+モジュールの項目で第5回目の講義動画をご視聴可能です。
 {{会員サイト}}
-＝＝＝＝＝＝＝
-第5回目の講義動画をご視聴ください。
-＜第5回目:オンライン化＞
-(動画本数・内容の詳細は、下書きに直接追記してください)
+＜第5回目の内容：（講義タイトル）＞
+（動画本数：X本）
+（動画①のタイトル（分）をここに追記）
+（動画②のタイトル（分））
+（動画③...）
+＜第5回目課題まとめは以下になります＞
+（課題①をここに追記）
+（課題② ※ブログチャレンジ、インスタチャレンジ等もここに）
+（課題③）
+講義動画ご視聴後は、
+{{期}}期のFBグループに第5回目講義のまとめも必ずご覧ください
 ━━━━━━━━━━━━━━━━━━━━━━
-【要挿入:Facebook投稿リンク】
-下記3つのFB投稿リンクを、送信前に貼り付けてください
+【要挿入：Facebook投稿リンク】
+下記2つのFB投稿リンクを、送信前に貼り付けてください
 ▼第5回目講義まとめ
-(URL挿入)
+（URL挿入）
 ▼課題をこなすための動画リンクなど
-(URL挿入)
-▼課題提出先リンクまとめ
-(URL挿入)
+（URL挿入）
 ━━━━━━━━━━━━━━━━━━━━━━
+【課題提出先リンクまとめ】
+{{課題提出先リンクまとめ}}
+※ご自身のお名前のシートをご自由にご活用ください。
 課題提出の期限は次回の講義動画配信日までとなっております。
+【次回の講座のグルコンの予定】
+（次回のグルコン予定をここに追記）
+ぜひご参加ください。
 ご案内は以上です。
 ご不明点のお問い合わせは
 当メールの返信にてご連絡ください。
@@ -1614,24 +1722,42 @@
           <t>※このメールは、『{{期}}期"Shine A Light"』の皆さまにお送りしております。
 こんにちは
 Shine A Light 運営事務局です。
-本日、第6回目の講義動画を会員サイトにアップいたしました。
+本日、第6回目の講義動画をお届けいたします。
+【第6回目の動画講義のご案内】
+第6回目の講義動画を会員サイトにアップしました。
+会員サイトよりご視聴ください。
 ＝＝＝＝＝＝＝
+第6回目講義動画「（講義タイトルをここに入れる）」
+＝＝＝＝＝＝＝
+会員サイトよりご視聴ください。
+モジュールの項目で第6回目の講義動画をご視聴可能です。
 {{会員サイト}}
-＝＝＝＝＝＝＝
-第6回目の講義動画をご視聴ください。
-＜第6回目:リピート・継続化＞
-(動画本数・内容の詳細は、下書きに直接追記してください)
+＜第6回目の内容：（講義タイトル）＞
+（動画本数：X本）
+（動画①のタイトル（分）をここに追記）
+（動画②のタイトル（分））
+（動画③...）
+＜第6回目課題まとめは以下になります＞
+（課題①をここに追記）
+（課題② ※ブログチャレンジ、インスタチャレンジ等もここに）
+（課題③）
+講義動画ご視聴後は、
+{{期}}期のFBグループに第6回目講義のまとめも必ずご覧ください
 ━━━━━━━━━━━━━━━━━━━━━━
-【要挿入:Facebook投稿リンク】
-下記3つのFB投稿リンクを、送信前に貼り付けてください
+【要挿入：Facebook投稿リンク】
+下記2つのFB投稿リンクを、送信前に貼り付けてください
 ▼第6回目講義まとめ
-(URL挿入)
+（URL挿入）
 ▼課題をこなすための動画リンクなど
-(URL挿入)
-▼課題提出先リンクまとめ
-(URL挿入)
+（URL挿入）
 ━━━━━━━━━━━━━━━━━━━━━━
+【課題提出先リンクまとめ】
+{{課題提出先リンクまとめ}}
+※ご自身のお名前のシートをご自由にご活用ください。
 課題提出の期限は次回の講義動画配信日までとなっております。
+【次回の講座のグルコンの予定】
+（次回のグルコン予定をここに追記）
+ぜひご参加ください。
 ご案内は以上です。
 ご不明点のお問い合わせは
 当メールの返信にてご連絡ください。

</xml_diff>

<commit_message>
Auto-fill next lecture and next キャッチアップウェンズデー in 動画配信 mails
New variables {{次回動画配信日}} and {{次回キャッチアップウェンズデー詳細}}
pulled from the スケジュール sheet at draft time: find the next matching
event after the current event.date. formatCatchupWedDetail combines
"6月17日（水）9時30分〜11時 神保麻紀先生". populateTemplate now takes
allEvents so it can search the schedule; buildBatchDrafts and processTargetDate
thread it through. Also merges the trigger setup helpers into Code.gs
(setupDailyTrigger / listTriggers / deleteDailyTrigger).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019MpwpoXeU7u2s8oySrLx9o
</commit_message>
<xml_diff>
--- a/scratchpad/MailTemplates_20ki_v2.xlsx
+++ b/scratchpad/MailTemplates_20ki_v2.xlsx
@@ -1430,8 +1430,11 @@
 {{課題提出先リンクまとめ}}
 ※ご自身のお名前のシートをご自由にご活用ください。
 課題提出の期限は次回の講義動画配信日までとなっております。
-【次回の講座のグルコンの予定】
-（次回のグルコン予定をここに追記）
+【次回の講義動画配信予定】
+{{次回動画配信日}}
+【次回のキャッチアップウェンズデー】
+キャッチアップウェンズデーグルコン（サポート講師担当）
+{{次回キャッチアップウェンズデー詳細}}の予定です。
 ぜひご参加ください。
 ご案内は以上です。
 ご不明点のお問い合わせは
@@ -1495,8 +1498,11 @@
 {{課題提出先リンクまとめ}}
 ※ご自身のお名前のシートをご自由にご活用ください。
 課題提出の期限は次回の講義動画配信日までとなっております。
-【次回の講座のグルコンの予定】
-（次回のグルコン予定をここに追記）
+【次回の講義動画配信予定】
+{{次回動画配信日}}
+【次回のキャッチアップウェンズデー】
+キャッチアップウェンズデーグルコン（サポート講師担当）
+{{次回キャッチアップウェンズデー詳細}}の予定です。
 ぜひご参加ください。
 ご案内は以上です。
 ご不明点のお問い合わせは
@@ -1560,8 +1566,11 @@
 {{課題提出先リンクまとめ}}
 ※ご自身のお名前のシートをご自由にご活用ください。
 課題提出の期限は次回の講義動画配信日までとなっております。
-【次回の講座のグルコンの予定】
-（次回のグルコン予定をここに追記）
+【次回の講義動画配信予定】
+{{次回動画配信日}}
+【次回のキャッチアップウェンズデー】
+キャッチアップウェンズデーグルコン（サポート講師担当）
+{{次回キャッチアップウェンズデー詳細}}の予定です。
 ぜひご参加ください。
 ご案内は以上です。
 ご不明点のお問い合わせは
@@ -1625,8 +1634,11 @@
 {{課題提出先リンクまとめ}}
 ※ご自身のお名前のシートをご自由にご活用ください。
 課題提出の期限は次回の講義動画配信日までとなっております。
-【次回の講座のグルコンの予定】
-（次回のグルコン予定をここに追記）
+【次回の講義動画配信予定】
+{{次回動画配信日}}
+【次回のキャッチアップウェンズデー】
+キャッチアップウェンズデーグルコン（サポート講師担当）
+{{次回キャッチアップウェンズデー詳細}}の予定です。
 ぜひご参加ください。
 ご案内は以上です。
 ご不明点のお問い合わせは
@@ -1690,8 +1702,11 @@
 {{課題提出先リンクまとめ}}
 ※ご自身のお名前のシートをご自由にご活用ください。
 課題提出の期限は次回の講義動画配信日までとなっております。
-【次回の講座のグルコンの予定】
-（次回のグルコン予定をここに追記）
+【次回の講義動画配信予定】
+{{次回動画配信日}}
+【次回のキャッチアップウェンズデー】
+キャッチアップウェンズデーグルコン（サポート講師担当）
+{{次回キャッチアップウェンズデー詳細}}の予定です。
 ぜひご参加ください。
 ご案内は以上です。
 ご不明点のお問い合わせは
@@ -1755,8 +1770,11 @@
 {{課題提出先リンクまとめ}}
 ※ご自身のお名前のシートをご自由にご活用ください。
 課題提出の期限は次回の講義動画配信日までとなっております。
-【次回の講座のグルコンの予定】
-（次回のグルコン予定をここに追記）
+【次回の講義動画配信予定】
+{{次回動画配信日}}
+【次回のキャッチアップウェンズデー】
+キャッチアップウェンズデーグルコン（サポート講師担当）
+{{次回キャッチアップウェンズデー詳細}}の予定です。
 ぜひご参加ください。
 ご案内は以上です。
 ご不明点のお問い合わせは

</xml_diff>